<commit_message>
updated hts prep and radet quartely pipelines
</commit_message>
<xml_diff>
--- a/csv_files/datatypes.xlsx
+++ b/csv_files/datatypes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\5300\Documents\Palladium\lamisplus_sync_ods_pipeline\csv_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6814CE04-2E87-4A03-91C3-6211225F550A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0CE6B61-8668-404C-B3CB-BF1374B2C679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{64222DD2-151F-4920-8B54-866558EEE237}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="datatypes" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">datatypes!$A$1:$A$1648</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">datatypes!$A$1:$A$1651</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5915" uniqueCount="851">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5927" uniqueCount="854">
   <si>
     <t>table_name</t>
   </si>
@@ -2576,6 +2576,15 @@
   </si>
   <si>
     <t>services_received_by_client</t>
+  </si>
+  <si>
+    <t>assessment_for_pep_indication</t>
+  </si>
+  <si>
+    <t>assessment_for_prep_eligibility</t>
+  </si>
+  <si>
+    <t>assessment_for_acute_hiv_infection</t>
   </si>
 </sst>
 </file>
@@ -3422,7 +3431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B6784D1-755D-4563-96EC-8753940C0388}">
-  <dimension ref="A1:E1648"/>
+  <dimension ref="A1:E1651"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="38.90625" style="1" bestFit="1" customWidth="1"/>
@@ -28309,13 +28318,13 @@
         <v>407</v>
       </c>
       <c r="B1464" s="1" t="s">
-        <v>408</v>
+        <v>851</v>
       </c>
       <c r="C1464" s="1" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="D1464" s="1">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="E1464" s="1" t="s">
         <v>8</v>
@@ -28326,13 +28335,13 @@
         <v>407</v>
       </c>
       <c r="B1465" s="1" t="s">
-        <v>101</v>
+        <v>852</v>
       </c>
       <c r="C1465" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D1465" s="1">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="E1465" s="1" t="s">
         <v>8</v>
@@ -28343,13 +28352,13 @@
         <v>407</v>
       </c>
       <c r="B1466" s="1" t="s">
-        <v>409</v>
+        <v>853</v>
       </c>
       <c r="C1466" s="1" t="s">
         <v>31</v>
       </c>
       <c r="D1466" s="1">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="E1466" s="1" t="s">
         <v>8</v>
@@ -28360,13 +28369,13 @@
         <v>407</v>
       </c>
       <c r="B1467" s="1" t="s">
-        <v>256</v>
+        <v>408</v>
       </c>
       <c r="C1467" s="1" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="D1467" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E1467" s="1" t="s">
         <v>8</v>
@@ -28377,13 +28386,13 @@
         <v>407</v>
       </c>
       <c r="B1468" s="1" t="s">
-        <v>410</v>
+        <v>101</v>
       </c>
       <c r="C1468" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D1468" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E1468" s="1" t="s">
         <v>8</v>
@@ -28394,13 +28403,13 @@
         <v>407</v>
       </c>
       <c r="B1469" s="1" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="C1469" s="1" t="s">
         <v>31</v>
       </c>
       <c r="D1469" s="1">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E1469" s="1" t="s">
         <v>8</v>
@@ -28411,13 +28420,13 @@
         <v>407</v>
       </c>
       <c r="B1470" s="1" t="s">
-        <v>412</v>
+        <v>256</v>
       </c>
       <c r="C1470" s="1" t="s">
         <v>31</v>
       </c>
       <c r="D1470" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E1470" s="1" t="s">
         <v>8</v>
@@ -28428,13 +28437,13 @@
         <v>407</v>
       </c>
       <c r="B1471" s="1" t="s">
-        <v>237</v>
+        <v>410</v>
       </c>
       <c r="C1471" s="1" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="D1471" s="1">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E1471" s="1" t="s">
         <v>8</v>
@@ -28445,13 +28454,13 @@
         <v>407</v>
       </c>
       <c r="B1472" s="1" t="s">
-        <v>239</v>
+        <v>411</v>
       </c>
       <c r="C1472" s="1" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="D1472" s="1">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E1472" s="1" t="s">
         <v>8</v>
@@ -28462,13 +28471,13 @@
         <v>407</v>
       </c>
       <c r="B1473" s="1" t="s">
-        <v>88</v>
+        <v>412</v>
       </c>
       <c r="C1473" s="1" t="s">
         <v>31</v>
       </c>
       <c r="D1473" s="1">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E1473" s="1" t="s">
         <v>8</v>
@@ -28479,13 +28488,13 @@
         <v>407</v>
       </c>
       <c r="B1474" s="1" t="s">
-        <v>84</v>
+        <v>237</v>
       </c>
       <c r="C1474" s="1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D1474" s="1">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E1474" s="1" t="s">
         <v>8</v>
@@ -28496,13 +28505,13 @@
         <v>407</v>
       </c>
       <c r="B1475" s="1" t="s">
-        <v>21</v>
+        <v>239</v>
       </c>
       <c r="C1475" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D1475" s="1">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E1475" s="1" t="s">
         <v>8</v>
@@ -28513,13 +28522,13 @@
         <v>407</v>
       </c>
       <c r="B1476" s="1" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="C1476" s="1" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="D1476" s="1">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E1476" s="1" t="s">
         <v>8</v>
@@ -28530,13 +28539,13 @@
         <v>407</v>
       </c>
       <c r="B1477" s="1" t="s">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="C1477" s="1" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D1477" s="1">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E1477" s="1" t="s">
         <v>8</v>
@@ -28547,13 +28556,13 @@
         <v>407</v>
       </c>
       <c r="B1478" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C1478" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D1478" s="1">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E1478" s="1" t="s">
         <v>8</v>
@@ -28564,16 +28573,16 @@
         <v>407</v>
       </c>
       <c r="B1479" s="1" t="s">
-        <v>147</v>
+        <v>19</v>
       </c>
       <c r="C1479" s="1" t="s">
-        <v>458</v>
+        <v>17</v>
       </c>
       <c r="D1479" s="1">
-        <v>2</v>
-      </c>
-      <c r="E1479" s="1">
-        <v>255</v>
+        <v>22</v>
+      </c>
+      <c r="E1479" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1480" spans="1:5" x14ac:dyDescent="0.35">
@@ -28581,13 +28590,13 @@
         <v>407</v>
       </c>
       <c r="B1480" s="1" t="s">
-        <v>512</v>
+        <v>20</v>
       </c>
       <c r="C1480" s="1" t="s">
-        <v>458</v>
+        <v>17</v>
       </c>
       <c r="D1480" s="1">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="E1480" s="1" t="s">
         <v>8</v>
@@ -28598,16 +28607,16 @@
         <v>407</v>
       </c>
       <c r="B1481" s="1" t="s">
-        <v>457</v>
+        <v>22</v>
       </c>
       <c r="C1481" s="1" t="s">
-        <v>458</v>
+        <v>11</v>
       </c>
       <c r="D1481" s="1">
-        <v>11</v>
-      </c>
-      <c r="E1481" s="1">
-        <v>255</v>
+        <v>1</v>
+      </c>
+      <c r="E1481" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1482" spans="1:5" x14ac:dyDescent="0.35">
@@ -28615,13 +28624,13 @@
         <v>407</v>
       </c>
       <c r="B1482" s="1" t="s">
-        <v>555</v>
+        <v>147</v>
       </c>
       <c r="C1482" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1482" s="1">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E1482" s="1">
         <v>255</v>
@@ -28632,16 +28641,16 @@
         <v>407</v>
       </c>
       <c r="B1483" s="1" t="s">
-        <v>556</v>
+        <v>512</v>
       </c>
       <c r="C1483" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1483" s="1">
-        <v>13</v>
-      </c>
-      <c r="E1483" s="1">
-        <v>255</v>
+        <v>3</v>
+      </c>
+      <c r="E1483" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1484" spans="1:5" x14ac:dyDescent="0.35">
@@ -28649,13 +28658,13 @@
         <v>407</v>
       </c>
       <c r="B1484" s="1" t="s">
-        <v>566</v>
+        <v>457</v>
       </c>
       <c r="C1484" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1484" s="1">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E1484" s="1">
         <v>255</v>
@@ -28666,13 +28675,13 @@
         <v>407</v>
       </c>
       <c r="B1485" s="1" t="s">
-        <v>502</v>
+        <v>555</v>
       </c>
       <c r="C1485" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1485" s="1">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E1485" s="1">
         <v>255</v>
@@ -28683,13 +28692,13 @@
         <v>407</v>
       </c>
       <c r="B1486" s="1" t="s">
-        <v>459</v>
+        <v>556</v>
       </c>
       <c r="C1486" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1486" s="1">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E1486" s="1">
         <v>255</v>
@@ -28700,13 +28709,13 @@
         <v>407</v>
       </c>
       <c r="B1487" s="1" t="s">
-        <v>460</v>
+        <v>566</v>
       </c>
       <c r="C1487" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1487" s="1">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="E1487" s="1">
         <v>255</v>
@@ -28714,53 +28723,53 @@
     </row>
     <row r="1488" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1488" s="1" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
       <c r="B1488" s="1" t="s">
-        <v>136</v>
+        <v>502</v>
       </c>
       <c r="C1488" s="1" t="s">
-        <v>28</v>
+        <v>458</v>
       </c>
       <c r="D1488" s="1">
-        <v>5</v>
-      </c>
-      <c r="E1488" s="1" t="s">
-        <v>8</v>
+        <v>17</v>
+      </c>
+      <c r="E1488" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1489" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1489" s="1" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
       <c r="B1489" s="1" t="s">
-        <v>88</v>
+        <v>459</v>
       </c>
       <c r="C1489" s="1" t="s">
-        <v>31</v>
+        <v>458</v>
       </c>
       <c r="D1489" s="1">
-        <v>8</v>
-      </c>
-      <c r="E1489" s="1" t="s">
-        <v>8</v>
+        <v>21</v>
+      </c>
+      <c r="E1489" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1490" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1490" s="1" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
       <c r="B1490" s="1" t="s">
-        <v>84</v>
+        <v>460</v>
       </c>
       <c r="C1490" s="1" t="s">
-        <v>11</v>
+        <v>458</v>
       </c>
       <c r="D1490" s="1">
-        <v>9</v>
-      </c>
-      <c r="E1490" s="1" t="s">
-        <v>8</v>
+        <v>23</v>
+      </c>
+      <c r="E1490" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1491" spans="1:5" x14ac:dyDescent="0.35">
@@ -28768,13 +28777,13 @@
         <v>413</v>
       </c>
       <c r="B1491" s="1" t="s">
-        <v>414</v>
+        <v>136</v>
       </c>
       <c r="C1491" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D1491" s="1">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E1491" s="1" t="s">
         <v>8</v>
@@ -28785,13 +28794,13 @@
         <v>413</v>
       </c>
       <c r="B1492" s="1" t="s">
-        <v>405</v>
+        <v>88</v>
       </c>
       <c r="C1492" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D1492" s="1">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E1492" s="1" t="s">
         <v>8</v>
@@ -28802,13 +28811,13 @@
         <v>413</v>
       </c>
       <c r="B1493" s="1" t="s">
-        <v>415</v>
+        <v>84</v>
       </c>
       <c r="C1493" s="1" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="D1493" s="1">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E1493" s="1" t="s">
         <v>8</v>
@@ -28819,13 +28828,13 @@
         <v>413</v>
       </c>
       <c r="B1494" s="1" t="s">
-        <v>21</v>
+        <v>414</v>
       </c>
       <c r="C1494" s="1" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="D1494" s="1">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E1494" s="1" t="s">
         <v>8</v>
@@ -28836,13 +28845,13 @@
         <v>413</v>
       </c>
       <c r="B1495" s="1" t="s">
-        <v>19</v>
+        <v>405</v>
       </c>
       <c r="C1495" s="1" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="D1495" s="1">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="E1495" s="1" t="s">
         <v>8</v>
@@ -28853,13 +28862,13 @@
         <v>413</v>
       </c>
       <c r="B1496" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="C1496" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1496" s="1">
         <v>20</v>
-      </c>
-      <c r="C1496" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1496" s="1">
-        <v>25</v>
       </c>
       <c r="E1496" s="1" t="s">
         <v>8</v>
@@ -28870,13 +28879,13 @@
         <v>413</v>
       </c>
       <c r="B1497" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C1497" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D1497" s="1">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="E1497" s="1" t="s">
         <v>8</v>
@@ -28887,16 +28896,16 @@
         <v>413</v>
       </c>
       <c r="B1498" s="1" t="s">
-        <v>512</v>
+        <v>19</v>
       </c>
       <c r="C1498" s="1" t="s">
-        <v>458</v>
+        <v>17</v>
       </c>
       <c r="D1498" s="1">
-        <v>2</v>
-      </c>
-      <c r="E1498" s="1">
-        <v>255</v>
+        <v>23</v>
+      </c>
+      <c r="E1498" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1499" spans="1:5" x14ac:dyDescent="0.35">
@@ -28904,16 +28913,16 @@
         <v>413</v>
       </c>
       <c r="B1499" s="1" t="s">
-        <v>502</v>
+        <v>20</v>
       </c>
       <c r="C1499" s="1" t="s">
-        <v>458</v>
+        <v>17</v>
       </c>
       <c r="D1499" s="1">
-        <v>3</v>
-      </c>
-      <c r="E1499" s="1">
-        <v>255</v>
+        <v>25</v>
+      </c>
+      <c r="E1499" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1500" spans="1:5" x14ac:dyDescent="0.35">
@@ -28921,16 +28930,16 @@
         <v>413</v>
       </c>
       <c r="B1500" s="1" t="s">
-        <v>147</v>
+        <v>22</v>
       </c>
       <c r="C1500" s="1" t="s">
-        <v>458</v>
+        <v>11</v>
       </c>
       <c r="D1500" s="1">
-        <v>4</v>
-      </c>
-      <c r="E1500" s="1">
-        <v>255</v>
+        <v>1</v>
+      </c>
+      <c r="E1500" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1501" spans="1:5" x14ac:dyDescent="0.35">
@@ -28938,13 +28947,13 @@
         <v>413</v>
       </c>
       <c r="B1501" s="1" t="s">
-        <v>457</v>
+        <v>512</v>
       </c>
       <c r="C1501" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1501" s="1">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E1501" s="1">
         <v>255</v>
@@ -28955,13 +28964,13 @@
         <v>413</v>
       </c>
       <c r="B1502" s="1" t="s">
-        <v>672</v>
+        <v>502</v>
       </c>
       <c r="C1502" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1502" s="1">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E1502" s="1">
         <v>255</v>
@@ -28972,16 +28981,16 @@
         <v>413</v>
       </c>
       <c r="B1503" s="1" t="s">
-        <v>699</v>
+        <v>147</v>
       </c>
       <c r="C1503" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1503" s="1">
-        <v>10</v>
-      </c>
-      <c r="E1503" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
+      </c>
+      <c r="E1503" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1504" spans="1:5" x14ac:dyDescent="0.35">
@@ -28989,16 +28998,16 @@
         <v>413</v>
       </c>
       <c r="B1504" s="1" t="s">
-        <v>66</v>
+        <v>457</v>
       </c>
       <c r="C1504" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1504" s="1">
-        <v>11</v>
-      </c>
-      <c r="E1504" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
+      </c>
+      <c r="E1504" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1505" spans="1:5" x14ac:dyDescent="0.35">
@@ -29006,16 +29015,16 @@
         <v>413</v>
       </c>
       <c r="B1505" s="1" t="s">
-        <v>741</v>
+        <v>672</v>
       </c>
       <c r="C1505" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1505" s="1">
-        <v>14</v>
-      </c>
-      <c r="E1505" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
+      </c>
+      <c r="E1505" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1506" spans="1:5" x14ac:dyDescent="0.35">
@@ -29023,13 +29032,13 @@
         <v>413</v>
       </c>
       <c r="B1506" s="1" t="s">
-        <v>745</v>
+        <v>699</v>
       </c>
       <c r="C1506" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1506" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E1506" s="1" t="s">
         <v>8</v>
@@ -29040,13 +29049,13 @@
         <v>413</v>
       </c>
       <c r="B1507" s="1" t="s">
-        <v>749</v>
+        <v>66</v>
       </c>
       <c r="C1507" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1507" s="1">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E1507" s="1" t="s">
         <v>8</v>
@@ -29057,13 +29066,13 @@
         <v>413</v>
       </c>
       <c r="B1508" s="1" t="s">
-        <v>754</v>
+        <v>741</v>
       </c>
       <c r="C1508" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1508" s="1">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E1508" s="1" t="s">
         <v>8</v>
@@ -29074,13 +29083,13 @@
         <v>413</v>
       </c>
       <c r="B1509" s="1" t="s">
-        <v>761</v>
+        <v>745</v>
       </c>
       <c r="C1509" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1509" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E1509" s="1" t="s">
         <v>8</v>
@@ -29091,13 +29100,13 @@
         <v>413</v>
       </c>
       <c r="B1510" s="1" t="s">
-        <v>765</v>
+        <v>749</v>
       </c>
       <c r="C1510" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1510" s="1">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E1510" s="1" t="s">
         <v>8</v>
@@ -29108,16 +29117,16 @@
         <v>413</v>
       </c>
       <c r="B1511" s="1" t="s">
-        <v>459</v>
+        <v>754</v>
       </c>
       <c r="C1511" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1511" s="1">
-        <v>22</v>
-      </c>
-      <c r="E1511" s="1">
-        <v>255</v>
+        <v>17</v>
+      </c>
+      <c r="E1511" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1512" spans="1:5" x14ac:dyDescent="0.35">
@@ -29125,30 +29134,30 @@
         <v>413</v>
       </c>
       <c r="B1512" s="1" t="s">
-        <v>460</v>
+        <v>761</v>
       </c>
       <c r="C1512" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1512" s="1">
-        <v>24</v>
-      </c>
-      <c r="E1512" s="1">
-        <v>255</v>
+        <v>18</v>
+      </c>
+      <c r="E1512" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1513" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1513" s="1" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="B1513" s="1" t="s">
-        <v>417</v>
+        <v>765</v>
       </c>
       <c r="C1513" s="1" t="s">
-        <v>28</v>
+        <v>458</v>
       </c>
       <c r="D1513" s="1">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="E1513" s="1" t="s">
         <v>8</v>
@@ -29156,36 +29165,36 @@
     </row>
     <row r="1514" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1514" s="1" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="B1514" s="1" t="s">
-        <v>418</v>
+        <v>459</v>
       </c>
       <c r="C1514" s="1" t="s">
-        <v>28</v>
+        <v>458</v>
       </c>
       <c r="D1514" s="1">
-        <v>7</v>
-      </c>
-      <c r="E1514" s="1" t="s">
-        <v>8</v>
+        <v>22</v>
+      </c>
+      <c r="E1514" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1515" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1515" s="1" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="B1515" s="1" t="s">
-        <v>419</v>
+        <v>460</v>
       </c>
       <c r="C1515" s="1" t="s">
-        <v>28</v>
+        <v>458</v>
       </c>
       <c r="D1515" s="1">
-        <v>10</v>
-      </c>
-      <c r="E1515" s="1" t="s">
-        <v>8</v>
+        <v>24</v>
+      </c>
+      <c r="E1515" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1516" spans="1:5" x14ac:dyDescent="0.35">
@@ -29193,13 +29202,13 @@
         <v>416</v>
       </c>
       <c r="B1516" s="1" t="s">
-        <v>88</v>
+        <v>417</v>
       </c>
       <c r="C1516" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D1516" s="1">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E1516" s="1" t="s">
         <v>8</v>
@@ -29210,13 +29219,13 @@
         <v>416</v>
       </c>
       <c r="B1517" s="1" t="s">
-        <v>84</v>
+        <v>418</v>
       </c>
       <c r="C1517" s="1" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="D1517" s="1">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E1517" s="1" t="s">
         <v>8</v>
@@ -29227,13 +29236,13 @@
         <v>416</v>
       </c>
       <c r="B1518" s="1" t="s">
-        <v>21</v>
+        <v>419</v>
       </c>
       <c r="C1518" s="1" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="D1518" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E1518" s="1" t="s">
         <v>8</v>
@@ -29244,13 +29253,13 @@
         <v>416</v>
       </c>
       <c r="B1519" s="1" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="C1519" s="1" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="D1519" s="1">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E1519" s="1" t="s">
         <v>8</v>
@@ -29261,13 +29270,13 @@
         <v>416</v>
       </c>
       <c r="B1520" s="1" t="s">
-        <v>420</v>
+        <v>84</v>
       </c>
       <c r="C1520" s="1" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="D1520" s="1">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E1520" s="1" t="s">
         <v>8</v>
@@ -29278,13 +29287,13 @@
         <v>416</v>
       </c>
       <c r="B1521" s="1" t="s">
-        <v>421</v>
+        <v>21</v>
       </c>
       <c r="C1521" s="1" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="D1521" s="1">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E1521" s="1" t="s">
         <v>8</v>
@@ -29295,13 +29304,13 @@
         <v>416</v>
       </c>
       <c r="B1522" s="1" t="s">
-        <v>422</v>
+        <v>19</v>
       </c>
       <c r="C1522" s="1" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D1522" s="1">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E1522" s="1" t="s">
         <v>8</v>
@@ -29312,13 +29321,13 @@
         <v>416</v>
       </c>
       <c r="B1523" s="1" t="s">
-        <v>339</v>
+        <v>420</v>
       </c>
       <c r="C1523" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D1523" s="1">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E1523" s="1" t="s">
         <v>8</v>
@@ -29329,13 +29338,13 @@
         <v>416</v>
       </c>
       <c r="B1524" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="C1524" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1524" s="1">
         <v>20</v>
-      </c>
-      <c r="C1524" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1524" s="1">
-        <v>23</v>
       </c>
       <c r="E1524" s="1" t="s">
         <v>8</v>
@@ -29346,13 +29355,13 @@
         <v>416</v>
       </c>
       <c r="B1525" s="1" t="s">
-        <v>22</v>
+        <v>422</v>
       </c>
       <c r="C1525" s="1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D1525" s="1">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="E1525" s="1" t="s">
         <v>8</v>
@@ -29363,16 +29372,16 @@
         <v>416</v>
       </c>
       <c r="B1526" s="1" t="s">
-        <v>459</v>
+        <v>339</v>
       </c>
       <c r="C1526" s="1" t="s">
-        <v>458</v>
+        <v>28</v>
       </c>
       <c r="D1526" s="1">
-        <v>16</v>
-      </c>
-      <c r="E1526" s="1">
-        <v>255</v>
+        <v>22</v>
+      </c>
+      <c r="E1526" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1527" spans="1:5" x14ac:dyDescent="0.35">
@@ -29380,16 +29389,16 @@
         <v>416</v>
       </c>
       <c r="B1527" s="1" t="s">
-        <v>460</v>
+        <v>20</v>
       </c>
       <c r="C1527" s="1" t="s">
-        <v>458</v>
+        <v>17</v>
       </c>
       <c r="D1527" s="1">
-        <v>18</v>
-      </c>
-      <c r="E1527" s="1">
-        <v>255</v>
+        <v>23</v>
+      </c>
+      <c r="E1527" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1528" spans="1:5" x14ac:dyDescent="0.35">
@@ -29397,13 +29406,13 @@
         <v>416</v>
       </c>
       <c r="B1528" s="1" t="s">
-        <v>466</v>
+        <v>22</v>
       </c>
       <c r="C1528" s="1" t="s">
-        <v>458</v>
+        <v>11</v>
       </c>
       <c r="D1528" s="1">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="E1528" s="1" t="s">
         <v>8</v>
@@ -29414,16 +29423,16 @@
         <v>416</v>
       </c>
       <c r="B1529" s="1" t="s">
-        <v>467</v>
+        <v>459</v>
       </c>
       <c r="C1529" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1529" s="1">
-        <v>25</v>
-      </c>
-      <c r="E1529" s="1" t="s">
-        <v>8</v>
+        <v>16</v>
+      </c>
+      <c r="E1529" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1530" spans="1:5" x14ac:dyDescent="0.35">
@@ -29431,13 +29440,13 @@
         <v>416</v>
       </c>
       <c r="B1530" s="1" t="s">
-        <v>147</v>
+        <v>460</v>
       </c>
       <c r="C1530" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1530" s="1">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="E1530" s="1">
         <v>255</v>
@@ -29448,16 +29457,16 @@
         <v>416</v>
       </c>
       <c r="B1531" s="1" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="C1531" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1531" s="1">
-        <v>3</v>
-      </c>
-      <c r="E1531" s="1">
-        <v>255</v>
+        <v>24</v>
+      </c>
+      <c r="E1531" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1532" spans="1:5" x14ac:dyDescent="0.35">
@@ -29465,16 +29474,16 @@
         <v>416</v>
       </c>
       <c r="B1532" s="1" t="s">
-        <v>790</v>
+        <v>467</v>
       </c>
       <c r="C1532" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1532" s="1">
-        <v>4</v>
-      </c>
-      <c r="E1532" s="1">
-        <v>255</v>
+        <v>25</v>
+      </c>
+      <c r="E1532" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1533" spans="1:5" x14ac:dyDescent="0.35">
@@ -29482,13 +29491,13 @@
         <v>416</v>
       </c>
       <c r="B1533" s="1" t="s">
-        <v>793</v>
+        <v>147</v>
       </c>
       <c r="C1533" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1533" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E1533" s="1">
         <v>255</v>
@@ -29499,13 +29508,13 @@
         <v>416</v>
       </c>
       <c r="B1534" s="1" t="s">
-        <v>798</v>
+        <v>457</v>
       </c>
       <c r="C1534" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1534" s="1">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E1534" s="1">
         <v>255</v>
@@ -29516,13 +29525,13 @@
         <v>416</v>
       </c>
       <c r="B1535" s="1" t="s">
-        <v>806</v>
+        <v>790</v>
       </c>
       <c r="C1535" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1535" s="1">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E1535" s="1">
         <v>255</v>
@@ -29533,13 +29542,13 @@
         <v>416</v>
       </c>
       <c r="B1536" s="1" t="s">
-        <v>811</v>
+        <v>793</v>
       </c>
       <c r="C1536" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1536" s="1">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E1536" s="1">
         <v>255</v>
@@ -29550,13 +29559,13 @@
         <v>416</v>
       </c>
       <c r="B1537" s="1" t="s">
-        <v>816</v>
+        <v>798</v>
       </c>
       <c r="C1537" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1537" s="1">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E1537" s="1">
         <v>255</v>
@@ -29564,53 +29573,53 @@
     </row>
     <row r="1538" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1538" s="1" t="s">
-        <v>423</v>
+        <v>416</v>
       </c>
       <c r="B1538" s="1" t="s">
-        <v>21</v>
+        <v>806</v>
       </c>
       <c r="C1538" s="1" t="s">
-        <v>14</v>
+        <v>458</v>
       </c>
       <c r="D1538" s="1">
-        <v>5</v>
-      </c>
-      <c r="E1538" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="E1538" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1539" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1539" s="1" t="s">
-        <v>423</v>
+        <v>416</v>
       </c>
       <c r="B1539" s="1" t="s">
-        <v>22</v>
+        <v>811</v>
       </c>
       <c r="C1539" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="D1539" s="1">
         <v>11</v>
       </c>
-      <c r="D1539" s="1">
-        <v>1</v>
-      </c>
-      <c r="E1539" s="1" t="s">
-        <v>8</v>
+      <c r="E1539" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1540" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1540" s="1" t="s">
-        <v>423</v>
+        <v>416</v>
       </c>
       <c r="B1540" s="1" t="s">
-        <v>477</v>
+        <v>816</v>
       </c>
       <c r="C1540" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1540" s="1">
-        <v>2</v>
-      </c>
-      <c r="E1540" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
+      </c>
+      <c r="E1540" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1541" spans="1:5" x14ac:dyDescent="0.35">
@@ -29618,13 +29627,13 @@
         <v>423</v>
       </c>
       <c r="B1541" s="1" t="s">
-        <v>484</v>
+        <v>21</v>
       </c>
       <c r="C1541" s="1" t="s">
-        <v>458</v>
+        <v>14</v>
       </c>
       <c r="D1541" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E1541" s="1" t="s">
         <v>8</v>
@@ -29635,13 +29644,13 @@
         <v>423</v>
       </c>
       <c r="B1542" s="1" t="s">
-        <v>483</v>
+        <v>22</v>
       </c>
       <c r="C1542" s="1" t="s">
-        <v>458</v>
+        <v>11</v>
       </c>
       <c r="D1542" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E1542" s="1" t="s">
         <v>8</v>
@@ -29652,13 +29661,13 @@
         <v>423</v>
       </c>
       <c r="B1543" s="1" t="s">
-        <v>321</v>
+        <v>477</v>
       </c>
       <c r="C1543" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1543" s="1">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E1543" s="1" t="s">
         <v>8</v>
@@ -29666,16 +29675,16 @@
     </row>
     <row r="1544" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1544" s="1" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B1544" s="1" t="s">
-        <v>22</v>
+        <v>484</v>
       </c>
       <c r="C1544" s="1" t="s">
-        <v>11</v>
+        <v>458</v>
       </c>
       <c r="D1544" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E1544" s="1" t="s">
         <v>8</v>
@@ -29683,16 +29692,16 @@
     </row>
     <row r="1545" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1545" s="1" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B1545" s="1" t="s">
-        <v>19</v>
+        <v>483</v>
       </c>
       <c r="C1545" s="1" t="s">
-        <v>17</v>
+        <v>458</v>
       </c>
       <c r="D1545" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E1545" s="1" t="s">
         <v>8</v>
@@ -29700,13 +29709,13 @@
     </row>
     <row r="1546" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1546" s="1" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B1546" s="1" t="s">
-        <v>425</v>
+        <v>321</v>
       </c>
       <c r="C1546" s="1" t="s">
-        <v>14</v>
+        <v>458</v>
       </c>
       <c r="D1546" s="1">
         <v>6</v>
@@ -29720,16 +29729,16 @@
         <v>424</v>
       </c>
       <c r="B1547" s="1" t="s">
-        <v>549</v>
+        <v>22</v>
       </c>
       <c r="C1547" s="1" t="s">
-        <v>458</v>
+        <v>11</v>
       </c>
       <c r="D1547" s="1">
-        <v>2</v>
-      </c>
-      <c r="E1547" s="1">
-        <v>255</v>
+        <v>1</v>
+      </c>
+      <c r="E1547" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1548" spans="1:5" x14ac:dyDescent="0.35">
@@ -29737,16 +29746,16 @@
         <v>424</v>
       </c>
       <c r="B1548" s="1" t="s">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="C1548" s="1" t="s">
-        <v>458</v>
+        <v>17</v>
       </c>
       <c r="D1548" s="1">
-        <v>3</v>
-      </c>
-      <c r="E1548" s="1">
-        <v>255</v>
+        <v>5</v>
+      </c>
+      <c r="E1548" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1549" spans="1:5" x14ac:dyDescent="0.35">
@@ -29754,16 +29763,16 @@
         <v>424</v>
       </c>
       <c r="B1549" s="1" t="s">
-        <v>552</v>
+        <v>425</v>
       </c>
       <c r="C1549" s="1" t="s">
-        <v>458</v>
+        <v>14</v>
       </c>
       <c r="D1549" s="1">
-        <v>4</v>
-      </c>
-      <c r="E1549" s="1">
-        <v>255</v>
+        <v>6</v>
+      </c>
+      <c r="E1549" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1550" spans="1:5" x14ac:dyDescent="0.35">
@@ -29771,13 +29780,13 @@
         <v>424</v>
       </c>
       <c r="B1550" s="1" t="s">
-        <v>66</v>
+        <v>549</v>
       </c>
       <c r="C1550" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1550" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E1550" s="1">
         <v>255</v>
@@ -29785,53 +29794,53 @@
     </row>
     <row r="1551" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1551" s="1" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="B1551" s="1" t="s">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="C1551" s="1" t="s">
-        <v>11</v>
+        <v>458</v>
       </c>
       <c r="D1551" s="1">
-        <v>6</v>
-      </c>
-      <c r="E1551" s="1" t="s">
-        <v>8</v>
+        <v>3</v>
+      </c>
+      <c r="E1551" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1552" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1552" s="1" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="B1552" s="1" t="s">
-        <v>34</v>
+        <v>552</v>
       </c>
       <c r="C1552" s="1" t="s">
-        <v>11</v>
+        <v>458</v>
       </c>
       <c r="D1552" s="1">
-        <v>7</v>
-      </c>
-      <c r="E1552" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
+      </c>
+      <c r="E1552" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1553" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1553" s="1" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="B1553" s="1" t="s">
-        <v>427</v>
+        <v>66</v>
       </c>
       <c r="C1553" s="1" t="s">
-        <v>11</v>
+        <v>458</v>
       </c>
       <c r="D1553" s="1">
-        <v>8</v>
-      </c>
-      <c r="E1553" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
+      </c>
+      <c r="E1553" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1554" spans="1:5" x14ac:dyDescent="0.35">
@@ -29839,13 +29848,13 @@
         <v>426</v>
       </c>
       <c r="B1554" s="1" t="s">
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="C1554" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D1554" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E1554" s="1" t="s">
         <v>8</v>
@@ -29856,13 +29865,13 @@
         <v>426</v>
       </c>
       <c r="B1555" s="1" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="C1555" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D1555" s="1">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E1555" s="1" t="s">
         <v>8</v>
@@ -29873,16 +29882,16 @@
         <v>426</v>
       </c>
       <c r="B1556" s="1" t="s">
-        <v>492</v>
+        <v>427</v>
       </c>
       <c r="C1556" s="1" t="s">
-        <v>458</v>
+        <v>11</v>
       </c>
       <c r="D1556" s="1">
-        <v>2</v>
-      </c>
-      <c r="E1556" s="1">
-        <v>255</v>
+        <v>8</v>
+      </c>
+      <c r="E1556" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1557" spans="1:5" x14ac:dyDescent="0.35">
@@ -29890,16 +29899,16 @@
         <v>426</v>
       </c>
       <c r="B1557" s="1" t="s">
-        <v>574</v>
+        <v>66</v>
       </c>
       <c r="C1557" s="1" t="s">
-        <v>458</v>
+        <v>11</v>
       </c>
       <c r="D1557" s="1">
-        <v>3</v>
-      </c>
-      <c r="E1557" s="1">
-        <v>10485760</v>
+        <v>12</v>
+      </c>
+      <c r="E1557" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1558" spans="1:5" x14ac:dyDescent="0.35">
@@ -29907,16 +29916,16 @@
         <v>426</v>
       </c>
       <c r="B1558" s="1" t="s">
-        <v>518</v>
+        <v>22</v>
       </c>
       <c r="C1558" s="1" t="s">
-        <v>458</v>
+        <v>11</v>
       </c>
       <c r="D1558" s="1">
-        <v>4</v>
-      </c>
-      <c r="E1558" s="1">
-        <v>255</v>
+        <v>1</v>
+      </c>
+      <c r="E1558" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1559" spans="1:5" x14ac:dyDescent="0.35">
@@ -29924,13 +29933,13 @@
         <v>426</v>
       </c>
       <c r="B1559" s="1" t="s">
-        <v>606</v>
+        <v>492</v>
       </c>
       <c r="C1559" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1559" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E1559" s="1">
         <v>255</v>
@@ -29941,13 +29950,13 @@
         <v>426</v>
       </c>
       <c r="B1560" s="1" t="s">
-        <v>643</v>
+        <v>574</v>
       </c>
       <c r="C1560" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1560" s="1">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E1560" s="1">
         <v>10485760</v>
@@ -29958,16 +29967,16 @@
         <v>426</v>
       </c>
       <c r="B1561" s="1" t="s">
-        <v>673</v>
+        <v>518</v>
       </c>
       <c r="C1561" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1561" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E1561" s="1">
-        <v>10485760</v>
+        <v>255</v>
       </c>
     </row>
     <row r="1562" spans="1:5" x14ac:dyDescent="0.35">
@@ -29975,81 +29984,81 @@
         <v>426</v>
       </c>
       <c r="B1562" s="1" t="s">
-        <v>682</v>
+        <v>606</v>
       </c>
       <c r="C1562" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1562" s="1">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E1562" s="1">
-        <v>10485760</v>
+        <v>255</v>
       </c>
     </row>
     <row r="1563" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1563" s="1" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="B1563" s="1" t="s">
-        <v>22</v>
+        <v>643</v>
       </c>
       <c r="C1563" s="1" t="s">
-        <v>11</v>
+        <v>458</v>
       </c>
       <c r="D1563" s="1">
-        <v>1</v>
-      </c>
-      <c r="E1563" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="E1563" s="1">
+        <v>10485760</v>
       </c>
     </row>
     <row r="1564" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1564" s="1" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="B1564" s="1" t="s">
-        <v>766</v>
+        <v>673</v>
       </c>
       <c r="C1564" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1564" s="1">
-        <v>2</v>
-      </c>
-      <c r="E1564" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="E1564" s="1">
+        <v>10485760</v>
       </c>
     </row>
     <row r="1565" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1565" s="1" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="B1565" s="1" t="s">
-        <v>147</v>
+        <v>682</v>
       </c>
       <c r="C1565" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1565" s="1">
-        <v>3</v>
-      </c>
-      <c r="E1565" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="E1565" s="1">
+        <v>10485760</v>
       </c>
     </row>
     <row r="1566" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1566" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B1566" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C1566" s="1" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="D1566" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E1566" s="1" t="s">
         <v>8</v>
@@ -30057,16 +30066,16 @@
     </row>
     <row r="1567" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1567" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B1567" s="1" t="s">
-        <v>22</v>
+        <v>766</v>
       </c>
       <c r="C1567" s="1" t="s">
-        <v>11</v>
+        <v>458</v>
       </c>
       <c r="D1567" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E1567" s="1" t="s">
         <v>8</v>
@@ -30074,16 +30083,16 @@
     </row>
     <row r="1568" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1568" s="1" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B1568" s="1" t="s">
-        <v>22</v>
+        <v>147</v>
       </c>
       <c r="C1568" s="1" t="s">
-        <v>147</v>
+        <v>458</v>
       </c>
       <c r="D1568" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E1568" s="1" t="s">
         <v>8</v>
@@ -30091,16 +30100,16 @@
     </row>
     <row r="1569" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1569" s="1" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B1569" s="1" t="s">
-        <v>431</v>
+        <v>30</v>
       </c>
       <c r="C1569" s="1" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="D1569" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E1569" s="1" t="s">
         <v>8</v>
@@ -30108,16 +30117,16 @@
     </row>
     <row r="1570" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1570" s="1" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B1570" s="1" t="s">
-        <v>432</v>
+        <v>22</v>
       </c>
       <c r="C1570" s="1" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D1570" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E1570" s="1" t="s">
         <v>8</v>
@@ -30128,13 +30137,13 @@
         <v>430</v>
       </c>
       <c r="B1571" s="1" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C1571" s="1" t="s">
-        <v>7</v>
+        <v>147</v>
       </c>
       <c r="D1571" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E1571" s="1" t="s">
         <v>8</v>
@@ -30145,16 +30154,16 @@
         <v>430</v>
       </c>
       <c r="B1572" s="1" t="s">
-        <v>507</v>
+        <v>431</v>
       </c>
       <c r="C1572" s="1" t="s">
-        <v>458</v>
+        <v>17</v>
       </c>
       <c r="D1572" s="1">
-        <v>2</v>
-      </c>
-      <c r="E1572" s="1">
-        <v>255</v>
+        <v>4</v>
+      </c>
+      <c r="E1572" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1573" spans="1:5" x14ac:dyDescent="0.35">
@@ -30162,30 +30171,30 @@
         <v>430</v>
       </c>
       <c r="B1573" s="1" t="s">
-        <v>16</v>
+        <v>432</v>
       </c>
       <c r="C1573" s="1" t="s">
-        <v>458</v>
+        <v>17</v>
       </c>
       <c r="D1573" s="1">
-        <v>3</v>
-      </c>
-      <c r="E1573" s="1">
-        <v>255</v>
+        <v>5</v>
+      </c>
+      <c r="E1573" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1574" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1574" s="1" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="B1574" s="1" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C1574" s="1" t="s">
-        <v>147</v>
+        <v>7</v>
       </c>
       <c r="D1574" s="1">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E1574" s="1" t="s">
         <v>8</v>
@@ -30193,33 +30202,33 @@
     </row>
     <row r="1575" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1575" s="1" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="B1575" s="1" t="s">
-        <v>434</v>
+        <v>507</v>
       </c>
       <c r="C1575" s="1" t="s">
-        <v>147</v>
+        <v>458</v>
       </c>
       <c r="D1575" s="1">
-        <v>4</v>
-      </c>
-      <c r="E1575" s="1" t="s">
-        <v>8</v>
+        <v>2</v>
+      </c>
+      <c r="E1575" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1576" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1576" s="1" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="B1576" s="1" t="s">
-        <v>462</v>
+        <v>16</v>
       </c>
       <c r="C1576" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1576" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1576" s="1">
         <v>255</v>
@@ -30230,30 +30239,30 @@
         <v>433</v>
       </c>
       <c r="B1577" s="1" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C1577" s="1" t="s">
-        <v>458</v>
+        <v>147</v>
       </c>
       <c r="D1577" s="1">
-        <v>3</v>
-      </c>
-      <c r="E1577" s="1">
-        <v>255</v>
+        <v>1</v>
+      </c>
+      <c r="E1577" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1578" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1578" s="1" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="B1578" s="1" t="s">
-        <v>22</v>
+        <v>434</v>
       </c>
       <c r="C1578" s="1" t="s">
         <v>147</v>
       </c>
       <c r="D1578" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E1578" s="1" t="s">
         <v>8</v>
@@ -30261,36 +30270,36 @@
     </row>
     <row r="1579" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1579" s="1" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="B1579" s="1" t="s">
-        <v>436</v>
+        <v>462</v>
       </c>
       <c r="C1579" s="1" t="s">
-        <v>147</v>
+        <v>458</v>
       </c>
       <c r="D1579" s="1">
-        <v>5</v>
-      </c>
-      <c r="E1579" s="1" t="s">
-        <v>8</v>
+        <v>2</v>
+      </c>
+      <c r="E1579" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1580" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1580" s="1" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="B1580" s="1" t="s">
-        <v>437</v>
+        <v>16</v>
       </c>
       <c r="C1580" s="1" t="s">
-        <v>7</v>
+        <v>458</v>
       </c>
       <c r="D1580" s="1">
-        <v>6</v>
-      </c>
-      <c r="E1580" s="1" t="s">
-        <v>8</v>
+        <v>3</v>
+      </c>
+      <c r="E1580" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1581" spans="1:5" x14ac:dyDescent="0.35">
@@ -30298,16 +30307,16 @@
         <v>435</v>
       </c>
       <c r="B1581" s="1" t="s">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="C1581" s="1" t="s">
-        <v>458</v>
+        <v>147</v>
       </c>
       <c r="D1581" s="1">
-        <v>2</v>
-      </c>
-      <c r="E1581" s="1">
-        <v>255</v>
+        <v>1</v>
+      </c>
+      <c r="E1581" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1582" spans="1:5" x14ac:dyDescent="0.35">
@@ -30315,16 +30324,16 @@
         <v>435</v>
       </c>
       <c r="B1582" s="1" t="s">
-        <v>475</v>
+        <v>436</v>
       </c>
       <c r="C1582" s="1" t="s">
-        <v>458</v>
+        <v>147</v>
       </c>
       <c r="D1582" s="1">
-        <v>3</v>
-      </c>
-      <c r="E1582" s="1">
-        <v>4000</v>
+        <v>5</v>
+      </c>
+      <c r="E1582" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1583" spans="1:5" x14ac:dyDescent="0.35">
@@ -30332,81 +30341,81 @@
         <v>435</v>
       </c>
       <c r="B1583" s="1" t="s">
-        <v>506</v>
+        <v>437</v>
       </c>
       <c r="C1583" s="1" t="s">
-        <v>458</v>
+        <v>7</v>
       </c>
       <c r="D1583" s="1">
-        <v>4</v>
-      </c>
-      <c r="E1583" s="1">
-        <v>255</v>
+        <v>6</v>
+      </c>
+      <c r="E1583" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1584" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1584" s="1" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="B1584" s="1" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="C1584" s="1" t="s">
-        <v>147</v>
+        <v>458</v>
       </c>
       <c r="D1584" s="1">
-        <v>1</v>
-      </c>
-      <c r="E1584" s="1" t="s">
-        <v>8</v>
+        <v>2</v>
+      </c>
+      <c r="E1584" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1585" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1585" s="1" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="B1585" s="1" t="s">
-        <v>84</v>
+        <v>475</v>
       </c>
       <c r="C1585" s="1" t="s">
-        <v>14</v>
+        <v>458</v>
       </c>
       <c r="D1585" s="1">
-        <v>2</v>
-      </c>
-      <c r="E1585" s="1" t="s">
-        <v>8</v>
+        <v>3</v>
+      </c>
+      <c r="E1585" s="1">
+        <v>4000</v>
       </c>
     </row>
     <row r="1586" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1586" s="1" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="B1586" s="1" t="s">
-        <v>611</v>
+        <v>506</v>
       </c>
       <c r="C1586" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1586" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1586" s="1">
-        <v>2000</v>
+        <v>255</v>
       </c>
     </row>
     <row r="1587" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1587" s="1" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B1587" s="1" t="s">
-        <v>440</v>
+        <v>22</v>
       </c>
       <c r="C1587" s="1" t="s">
-        <v>17</v>
+        <v>147</v>
       </c>
       <c r="D1587" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E1587" s="1" t="s">
         <v>8</v>
@@ -30414,16 +30423,16 @@
     </row>
     <row r="1588" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1588" s="1" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B1588" s="1" t="s">
-        <v>34</v>
+        <v>84</v>
       </c>
       <c r="C1588" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D1588" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E1588" s="1" t="s">
         <v>8</v>
@@ -30431,19 +30440,19 @@
     </row>
     <row r="1589" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1589" s="1" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B1589" s="1" t="s">
-        <v>441</v>
+        <v>611</v>
       </c>
       <c r="C1589" s="1" t="s">
-        <v>14</v>
+        <v>458</v>
       </c>
       <c r="D1589" s="1">
-        <v>5</v>
-      </c>
-      <c r="E1589" s="1" t="s">
-        <v>8</v>
+        <v>3</v>
+      </c>
+      <c r="E1589" s="1">
+        <v>2000</v>
       </c>
     </row>
     <row r="1590" spans="1:5" x14ac:dyDescent="0.35">
@@ -30451,13 +30460,13 @@
         <v>439</v>
       </c>
       <c r="B1590" s="1" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="C1590" s="1" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D1590" s="1">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E1590" s="1" t="s">
         <v>8</v>
@@ -30468,13 +30477,13 @@
         <v>439</v>
       </c>
       <c r="B1591" s="1" t="s">
-        <v>443</v>
+        <v>34</v>
       </c>
       <c r="C1591" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D1591" s="1">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E1591" s="1" t="s">
         <v>8</v>
@@ -30485,13 +30494,13 @@
         <v>439</v>
       </c>
       <c r="B1592" s="1" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="C1592" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D1592" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E1592" s="1" t="s">
         <v>8</v>
@@ -30502,13 +30511,13 @@
         <v>439</v>
       </c>
       <c r="B1593" s="1" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="C1593" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D1593" s="1">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E1593" s="1" t="s">
         <v>8</v>
@@ -30519,13 +30528,13 @@
         <v>439</v>
       </c>
       <c r="B1594" s="1" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="C1594" s="1" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="D1594" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E1594" s="1" t="s">
         <v>8</v>
@@ -30536,13 +30545,13 @@
         <v>439</v>
       </c>
       <c r="B1595" s="1" t="s">
-        <v>22</v>
+        <v>444</v>
       </c>
       <c r="C1595" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D1595" s="1">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E1595" s="1" t="s">
         <v>8</v>
@@ -30553,16 +30562,16 @@
         <v>439</v>
       </c>
       <c r="B1596" s="1" t="s">
-        <v>0</v>
+        <v>445</v>
       </c>
       <c r="C1596" s="1" t="s">
-        <v>458</v>
+        <v>14</v>
       </c>
       <c r="D1596" s="1">
-        <v>4</v>
-      </c>
-      <c r="E1596" s="1">
-        <v>255</v>
+        <v>9</v>
+      </c>
+      <c r="E1596" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1597" spans="1:5" x14ac:dyDescent="0.35">
@@ -30570,13 +30579,13 @@
         <v>439</v>
       </c>
       <c r="B1597" s="1" t="s">
-        <v>819</v>
+        <v>446</v>
       </c>
       <c r="C1597" s="1" t="s">
-        <v>458</v>
+        <v>31</v>
       </c>
       <c r="D1597" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E1597" s="1" t="s">
         <v>8</v>
@@ -30584,16 +30593,16 @@
     </row>
     <row r="1598" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1598" s="1" t="s">
-        <v>447</v>
+        <v>439</v>
       </c>
       <c r="B1598" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C1598" s="1" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D1598" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E1598" s="1" t="s">
         <v>8</v>
@@ -30601,33 +30610,33 @@
     </row>
     <row r="1599" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1599" s="1" t="s">
-        <v>447</v>
+        <v>439</v>
       </c>
       <c r="B1599" s="1" t="s">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="C1599" s="1" t="s">
-        <v>11</v>
+        <v>458</v>
       </c>
       <c r="D1599" s="1">
         <v>4</v>
       </c>
-      <c r="E1599" s="1" t="s">
-        <v>8</v>
+      <c r="E1599" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1600" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1600" s="1" t="s">
-        <v>447</v>
+        <v>439</v>
       </c>
       <c r="B1600" s="1" t="s">
-        <v>441</v>
+        <v>819</v>
       </c>
       <c r="C1600" s="1" t="s">
-        <v>14</v>
+        <v>458</v>
       </c>
       <c r="D1600" s="1">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E1600" s="1" t="s">
         <v>8</v>
@@ -30638,13 +30647,13 @@
         <v>447</v>
       </c>
       <c r="B1601" s="1" t="s">
-        <v>444</v>
+        <v>19</v>
       </c>
       <c r="C1601" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D1601" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E1601" s="1" t="s">
         <v>8</v>
@@ -30655,13 +30664,13 @@
         <v>447</v>
       </c>
       <c r="B1602" s="1" t="s">
-        <v>445</v>
+        <v>34</v>
       </c>
       <c r="C1602" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D1602" s="1">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E1602" s="1" t="s">
         <v>8</v>
@@ -30672,13 +30681,13 @@
         <v>447</v>
       </c>
       <c r="B1603" s="1" t="s">
-        <v>448</v>
+        <v>441</v>
       </c>
       <c r="C1603" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D1603" s="1">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E1603" s="1" t="s">
         <v>8</v>
@@ -30689,13 +30698,13 @@
         <v>447</v>
       </c>
       <c r="B1604" s="1" t="s">
-        <v>22</v>
+        <v>444</v>
       </c>
       <c r="C1604" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D1604" s="1">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E1604" s="1" t="s">
         <v>8</v>
@@ -30706,16 +30715,16 @@
         <v>447</v>
       </c>
       <c r="B1605" s="1" t="s">
-        <v>465</v>
+        <v>445</v>
       </c>
       <c r="C1605" s="1" t="s">
-        <v>458</v>
+        <v>14</v>
       </c>
       <c r="D1605" s="1">
-        <v>3</v>
-      </c>
-      <c r="E1605" s="1">
-        <v>255</v>
+        <v>8</v>
+      </c>
+      <c r="E1605" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1606" spans="1:5" x14ac:dyDescent="0.35">
@@ -30723,16 +30732,16 @@
         <v>447</v>
       </c>
       <c r="B1606" s="1" t="s">
-        <v>0</v>
+        <v>448</v>
       </c>
       <c r="C1606" s="1" t="s">
-        <v>458</v>
+        <v>14</v>
       </c>
       <c r="D1606" s="1">
-        <v>6</v>
-      </c>
-      <c r="E1606" s="1">
-        <v>255</v>
+        <v>9</v>
+      </c>
+      <c r="E1606" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1607" spans="1:5" x14ac:dyDescent="0.35">
@@ -30740,13 +30749,13 @@
         <v>447</v>
       </c>
       <c r="B1607" s="1" t="s">
-        <v>459</v>
+        <v>22</v>
       </c>
       <c r="C1607" s="1" t="s">
-        <v>458</v>
+        <v>11</v>
       </c>
       <c r="D1607" s="1">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E1607" s="1" t="s">
         <v>8</v>
@@ -30754,53 +30763,53 @@
     </row>
     <row r="1608" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1608" s="1" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B1608" s="1" t="s">
-        <v>84</v>
+        <v>465</v>
       </c>
       <c r="C1608" s="1" t="s">
-        <v>11</v>
+        <v>458</v>
       </c>
       <c r="D1608" s="1">
-        <v>2</v>
-      </c>
-      <c r="E1608" s="1" t="s">
-        <v>8</v>
+        <v>3</v>
+      </c>
+      <c r="E1608" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1609" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1609" s="1" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B1609" s="1" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="C1609" s="1" t="s">
-        <v>11</v>
+        <v>458</v>
       </c>
       <c r="D1609" s="1">
-        <v>1</v>
-      </c>
-      <c r="E1609" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
+      </c>
+      <c r="E1609" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1610" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1610" s="1" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B1610" s="1" t="s">
-        <v>772</v>
+        <v>459</v>
       </c>
       <c r="C1610" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1610" s="1">
-        <v>3</v>
-      </c>
-      <c r="E1610" s="1">
-        <v>255</v>
+        <v>10</v>
+      </c>
+      <c r="E1610" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1611" spans="1:5" x14ac:dyDescent="0.35">
@@ -30808,16 +30817,16 @@
         <v>449</v>
       </c>
       <c r="B1611" s="1" t="s">
-        <v>773</v>
+        <v>84</v>
       </c>
       <c r="C1611" s="1" t="s">
-        <v>458</v>
+        <v>11</v>
       </c>
       <c r="D1611" s="1">
-        <v>4</v>
-      </c>
-      <c r="E1611" s="1">
-        <v>255</v>
+        <v>2</v>
+      </c>
+      <c r="E1611" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1612" spans="1:5" x14ac:dyDescent="0.35">
@@ -30825,67 +30834,67 @@
         <v>449</v>
       </c>
       <c r="B1612" s="1" t="s">
-        <v>774</v>
+        <v>22</v>
       </c>
       <c r="C1612" s="1" t="s">
-        <v>458</v>
+        <v>11</v>
       </c>
       <c r="D1612" s="1">
-        <v>5</v>
-      </c>
-      <c r="E1612" s="1">
-        <v>255</v>
+        <v>1</v>
+      </c>
+      <c r="E1612" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1613" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1613" s="1" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B1613" s="1" t="s">
-        <v>82</v>
+        <v>772</v>
       </c>
       <c r="C1613" s="1" t="s">
-        <v>17</v>
+        <v>458</v>
       </c>
       <c r="D1613" s="1">
-        <v>2</v>
-      </c>
-      <c r="E1613" s="1" t="s">
-        <v>8</v>
+        <v>3</v>
+      </c>
+      <c r="E1613" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1614" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1614" s="1" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B1614" s="1" t="s">
-        <v>83</v>
+        <v>773</v>
       </c>
       <c r="C1614" s="1" t="s">
-        <v>17</v>
+        <v>458</v>
       </c>
       <c r="D1614" s="1">
         <v>4</v>
       </c>
-      <c r="E1614" s="1" t="s">
-        <v>8</v>
+      <c r="E1614" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1615" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1615" s="1" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B1615" s="1" t="s">
-        <v>84</v>
+        <v>774</v>
       </c>
       <c r="C1615" s="1" t="s">
-        <v>11</v>
+        <v>458</v>
       </c>
       <c r="D1615" s="1">
-        <v>6</v>
-      </c>
-      <c r="E1615" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
+      </c>
+      <c r="E1615" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1616" spans="1:5" x14ac:dyDescent="0.35">
@@ -30893,13 +30902,13 @@
         <v>450</v>
       </c>
       <c r="B1616" s="1" t="s">
-        <v>152</v>
+        <v>82</v>
       </c>
       <c r="C1616" s="1" t="s">
-        <v>125</v>
+        <v>17</v>
       </c>
       <c r="D1616" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E1616" s="1" t="s">
         <v>8</v>
@@ -30910,13 +30919,13 @@
         <v>450</v>
       </c>
       <c r="B1617" s="1" t="s">
-        <v>153</v>
+        <v>83</v>
       </c>
       <c r="C1617" s="1" t="s">
-        <v>125</v>
+        <v>17</v>
       </c>
       <c r="D1617" s="1">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E1617" s="1" t="s">
         <v>8</v>
@@ -30927,13 +30936,13 @@
         <v>450</v>
       </c>
       <c r="B1618" s="1" t="s">
-        <v>156</v>
+        <v>84</v>
       </c>
       <c r="C1618" s="1" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D1618" s="1">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E1618" s="1" t="s">
         <v>8</v>
@@ -30944,13 +30953,13 @@
         <v>450</v>
       </c>
       <c r="B1619" s="1" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C1619" s="1" t="s">
         <v>125</v>
       </c>
       <c r="D1619" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E1619" s="1" t="s">
         <v>8</v>
@@ -30961,13 +30970,13 @@
         <v>450</v>
       </c>
       <c r="B1620" s="1" t="s">
-        <v>392</v>
+        <v>153</v>
       </c>
       <c r="C1620" s="1" t="s">
         <v>125</v>
       </c>
       <c r="D1620" s="1">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E1620" s="1" t="s">
         <v>8</v>
@@ -30978,13 +30987,13 @@
         <v>450</v>
       </c>
       <c r="B1621" s="1" t="s">
-        <v>391</v>
+        <v>156</v>
       </c>
       <c r="C1621" s="1" t="s">
-        <v>125</v>
+        <v>17</v>
       </c>
       <c r="D1621" s="1">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E1621" s="1" t="s">
         <v>8</v>
@@ -30995,13 +31004,13 @@
         <v>450</v>
       </c>
       <c r="B1622" s="1" t="s">
-        <v>393</v>
+        <v>155</v>
       </c>
       <c r="C1622" s="1" t="s">
         <v>125</v>
       </c>
       <c r="D1622" s="1">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E1622" s="1" t="s">
         <v>8</v>
@@ -31012,13 +31021,13 @@
         <v>450</v>
       </c>
       <c r="B1623" s="1" t="s">
-        <v>154</v>
+        <v>392</v>
       </c>
       <c r="C1623" s="1" t="s">
         <v>125</v>
       </c>
       <c r="D1623" s="1">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E1623" s="1" t="s">
         <v>8</v>
@@ -31029,13 +31038,13 @@
         <v>450</v>
       </c>
       <c r="B1624" s="1" t="s">
-        <v>21</v>
+        <v>391</v>
       </c>
       <c r="C1624" s="1" t="s">
-        <v>14</v>
+        <v>125</v>
       </c>
       <c r="D1624" s="1">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E1624" s="1" t="s">
         <v>8</v>
@@ -31046,13 +31055,13 @@
         <v>450</v>
       </c>
       <c r="B1625" s="1" t="s">
-        <v>22</v>
+        <v>393</v>
       </c>
       <c r="C1625" s="1" t="s">
-        <v>11</v>
+        <v>125</v>
       </c>
       <c r="D1625" s="1">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E1625" s="1" t="s">
         <v>8</v>
@@ -31063,16 +31072,16 @@
         <v>450</v>
       </c>
       <c r="B1626" s="1" t="s">
-        <v>459</v>
+        <v>154</v>
       </c>
       <c r="C1626" s="1" t="s">
-        <v>458</v>
+        <v>125</v>
       </c>
       <c r="D1626" s="1">
-        <v>3</v>
-      </c>
-      <c r="E1626" s="1">
-        <v>255</v>
+        <v>16</v>
+      </c>
+      <c r="E1626" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1627" spans="1:5" x14ac:dyDescent="0.35">
@@ -31080,16 +31089,16 @@
         <v>450</v>
       </c>
       <c r="B1627" s="1" t="s">
-        <v>464</v>
+        <v>21</v>
       </c>
       <c r="C1627" s="1" t="s">
-        <v>458</v>
+        <v>14</v>
       </c>
       <c r="D1627" s="1">
-        <v>5</v>
-      </c>
-      <c r="E1627" s="1">
-        <v>255</v>
+        <v>17</v>
+      </c>
+      <c r="E1627" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1628" spans="1:5" x14ac:dyDescent="0.35">
@@ -31097,16 +31106,16 @@
         <v>450</v>
       </c>
       <c r="B1628" s="1" t="s">
-        <v>457</v>
+        <v>22</v>
       </c>
       <c r="C1628" s="1" t="s">
-        <v>458</v>
+        <v>11</v>
       </c>
       <c r="D1628" s="1">
-        <v>14</v>
-      </c>
-      <c r="E1628" s="1">
-        <v>255</v>
+        <v>1</v>
+      </c>
+      <c r="E1628" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1629" spans="1:5" x14ac:dyDescent="0.35">
@@ -31114,13 +31123,13 @@
         <v>450</v>
       </c>
       <c r="B1629" s="1" t="s">
-        <v>110</v>
+        <v>459</v>
       </c>
       <c r="C1629" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1629" s="1">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E1629" s="1">
         <v>255</v>
@@ -31131,13 +31140,13 @@
         <v>450</v>
       </c>
       <c r="B1630" s="1" t="s">
-        <v>147</v>
+        <v>464</v>
       </c>
       <c r="C1630" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1630" s="1">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="E1630" s="1">
         <v>255</v>
@@ -31145,53 +31154,53 @@
     </row>
     <row r="1631" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1631" s="1" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B1631" s="1" t="s">
-        <v>22</v>
+        <v>457</v>
       </c>
       <c r="C1631" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="D1631" s="1">
         <v>14</v>
       </c>
-      <c r="D1631" s="1">
-        <v>1</v>
-      </c>
-      <c r="E1631" s="1" t="s">
-        <v>8</v>
+      <c r="E1631" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1632" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1632" s="1" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B1632" s="1" t="s">
-        <v>84</v>
+        <v>110</v>
       </c>
       <c r="C1632" s="1" t="s">
-        <v>14</v>
+        <v>458</v>
       </c>
       <c r="D1632" s="1">
-        <v>3</v>
-      </c>
-      <c r="E1632" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
+      </c>
+      <c r="E1632" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1633" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1633" s="1" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B1633" s="1" t="s">
-        <v>82</v>
+        <v>147</v>
       </c>
       <c r="C1633" s="1" t="s">
-        <v>17</v>
+        <v>458</v>
       </c>
       <c r="D1633" s="1">
-        <v>4</v>
-      </c>
-      <c r="E1633" s="1" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="E1633" s="1">
+        <v>255</v>
       </c>
     </row>
     <row r="1634" spans="1:5" x14ac:dyDescent="0.35">
@@ -31199,13 +31208,13 @@
         <v>451</v>
       </c>
       <c r="B1634" s="1" t="s">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="C1634" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D1634" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E1634" s="1" t="s">
         <v>8</v>
@@ -31216,13 +31225,13 @@
         <v>451</v>
       </c>
       <c r="B1635" s="1" t="s">
-        <v>21</v>
+        <v>84</v>
       </c>
       <c r="C1635" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D1635" s="1">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E1635" s="1" t="s">
         <v>8</v>
@@ -31233,13 +31242,13 @@
         <v>451</v>
       </c>
       <c r="B1636" s="1" t="s">
-        <v>152</v>
+        <v>82</v>
       </c>
       <c r="C1636" s="1" t="s">
-        <v>125</v>
+        <v>17</v>
       </c>
       <c r="D1636" s="1">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E1636" s="1" t="s">
         <v>8</v>
@@ -31250,13 +31259,13 @@
         <v>451</v>
       </c>
       <c r="B1637" s="1" t="s">
-        <v>153</v>
+        <v>83</v>
       </c>
       <c r="C1637" s="1" t="s">
-        <v>125</v>
+        <v>17</v>
       </c>
       <c r="D1637" s="1">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E1637" s="1" t="s">
         <v>8</v>
@@ -31267,13 +31276,13 @@
         <v>451</v>
       </c>
       <c r="B1638" s="1" t="s">
-        <v>154</v>
+        <v>21</v>
       </c>
       <c r="C1638" s="1" t="s">
-        <v>125</v>
+        <v>14</v>
       </c>
       <c r="D1638" s="1">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E1638" s="1" t="s">
         <v>8</v>
@@ -31284,13 +31293,13 @@
         <v>451</v>
       </c>
       <c r="B1639" s="1" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C1639" s="1" t="s">
         <v>125</v>
       </c>
       <c r="D1639" s="1">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E1639" s="1" t="s">
         <v>8</v>
@@ -31301,13 +31310,13 @@
         <v>451</v>
       </c>
       <c r="B1640" s="1" t="s">
-        <v>392</v>
+        <v>153</v>
       </c>
       <c r="C1640" s="1" t="s">
         <v>125</v>
       </c>
       <c r="D1640" s="1">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E1640" s="1" t="s">
         <v>8</v>
@@ -31318,13 +31327,13 @@
         <v>451</v>
       </c>
       <c r="B1641" s="1" t="s">
-        <v>391</v>
+        <v>154</v>
       </c>
       <c r="C1641" s="1" t="s">
         <v>125</v>
       </c>
       <c r="D1641" s="1">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E1641" s="1" t="s">
         <v>8</v>
@@ -31335,13 +31344,13 @@
         <v>451</v>
       </c>
       <c r="B1642" s="1" t="s">
-        <v>393</v>
+        <v>155</v>
       </c>
       <c r="C1642" s="1" t="s">
         <v>125</v>
       </c>
       <c r="D1642" s="1">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E1642" s="1" t="s">
         <v>8</v>
@@ -31352,13 +31361,13 @@
         <v>451</v>
       </c>
       <c r="B1643" s="1" t="s">
-        <v>156</v>
+        <v>392</v>
       </c>
       <c r="C1643" s="1" t="s">
-        <v>17</v>
+        <v>125</v>
       </c>
       <c r="D1643" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E1643" s="1" t="s">
         <v>8</v>
@@ -31369,16 +31378,16 @@
         <v>451</v>
       </c>
       <c r="B1644" s="1" t="s">
-        <v>457</v>
+        <v>391</v>
       </c>
       <c r="C1644" s="1" t="s">
-        <v>458</v>
+        <v>125</v>
       </c>
       <c r="D1644" s="1">
-        <v>2</v>
-      </c>
-      <c r="E1644" s="1">
-        <v>230</v>
+        <v>16</v>
+      </c>
+      <c r="E1644" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1645" spans="1:5" x14ac:dyDescent="0.35">
@@ -31386,16 +31395,16 @@
         <v>451</v>
       </c>
       <c r="B1645" s="1" t="s">
-        <v>464</v>
+        <v>393</v>
       </c>
       <c r="C1645" s="1" t="s">
-        <v>458</v>
+        <v>125</v>
       </c>
       <c r="D1645" s="1">
-        <v>7</v>
-      </c>
-      <c r="E1645" s="1">
-        <v>239</v>
+        <v>17</v>
+      </c>
+      <c r="E1645" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="1646" spans="1:5" x14ac:dyDescent="0.35">
@@ -31403,13 +31412,13 @@
         <v>451</v>
       </c>
       <c r="B1646" s="1" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="C1646" s="1" t="s">
-        <v>458</v>
+        <v>17</v>
       </c>
       <c r="D1646" s="1">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="E1646" s="1" t="s">
         <v>8</v>
@@ -31420,16 +31429,16 @@
         <v>451</v>
       </c>
       <c r="B1647" s="1" t="s">
-        <v>110</v>
+        <v>457</v>
       </c>
       <c r="C1647" s="1" t="s">
         <v>458</v>
       </c>
       <c r="D1647" s="1">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E1647" s="1">
-        <v>50</v>
+        <v>230</v>
       </c>
     </row>
     <row r="1648" spans="1:5" x14ac:dyDescent="0.35">
@@ -31437,21 +31446,72 @@
         <v>451</v>
       </c>
       <c r="B1648" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="C1648" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="D1648" s="1">
+        <v>7</v>
+      </c>
+      <c r="E1648" s="1">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="1649" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1649" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="B1649" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C1649" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="D1649" s="1">
+        <v>8</v>
+      </c>
+      <c r="E1649" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1650" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1650" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="B1650" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C1650" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="D1650" s="1">
+        <v>9</v>
+      </c>
+      <c r="E1650" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1651" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1651" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="B1651" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="C1648" s="1" t="s">
-        <v>458</v>
-      </c>
-      <c r="D1648" s="1">
+      <c r="C1651" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="D1651" s="1">
         <v>6</v>
       </c>
-      <c r="E1648" s="1">
+      <c r="E1651" s="1">
         <v>230</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E1648">
-    <sortCondition ref="A1:A1648"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E1651">
+    <sortCondition ref="A1:A1651"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>